<commit_message>
Redesign course cards with module bullets and link-based interest tracking
</commit_message>
<xml_diff>
--- a/data/courses_data.xlsx
+++ b/data/courses_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="176">
   <si>
     <t>program</t>
   </si>
@@ -28,6 +28,9 @@
     <t>description</t>
   </si>
   <si>
+    <t>modules</t>
+  </si>
+  <si>
     <t>urlslug</t>
   </si>
   <si>
@@ -266,6 +269,96 @@
   </si>
   <si>
     <t>Covers Digital Marketing Foundations &amp; Strategy, SEO Specialist Track, Website Development &amp; Landing Pages, Social Media Marketing &amp; Management, Content Marketing &amp; Copywriting, plus 7 more modules, building practical, job-ready skills in Advanced Digital Marketing Performance.</t>
+  </si>
+  <si>
+    <t>Frontend (Figma, HTML, CSS, JavaScript); Backend (Core &amp; Advance Python); Frontend Library (React. JS); Framework (Django with REST (DRF) API); Git &amp; SDLC; Data Structures &amp; Algorithms (Python); Machine Learning (Supervised &amp; Unsupervised); Artificial Intelligence; Database (MySQL); Python Libraries(Numpy, Pandas, Matplotlib, Seaborn); Data Visualization (Power BI); Cloud (Azure)</t>
+  </si>
+  <si>
+    <t>Figma, HTML, CSS, JavaScript; Backend (Core &amp; Advance Python); Frontend Library (React. JS); Framework (Django with REST (DRF) API); Git &amp; SDLC; Data Structures &amp; Algorithms (Python); Mobile App (Flutter)</t>
+  </si>
+  <si>
+    <t>Frontend (Figma, HTML, CSS, JavaScript); Database (Mongo DB); Frontend Library (React. JS); Framework (Node js with REST API); Git &amp; SDLC; Mobile App (React Native)</t>
+  </si>
+  <si>
+    <t>Adv Excel with Dashboard; Statistics &amp; Mathematics for Data Analytics</t>
+  </si>
+  <si>
+    <t>Frontend (Figma, HTML, CSS, JavaScript); Backend (Core &amp; Advance Python); Frontend Library (React. JS); Framework (Django with REST (DRF) API); Git &amp; SDLC; Data Structures &amp; Algorithms (Python); Machine Learning (Supervised &amp; Unsupervised); Artificial Intelligence; Database (MySQL); Python Libraries(Numpy, Pandas, Matplotlib, Seaborn); Data Visualization (Power BI); Cloud (Azure); Mobile App (Flutter)</t>
+  </si>
+  <si>
+    <t>Frontend (Figma, HTML, CSS, JavaScript); Backend (Core &amp; Advance Python); Frontend Library (React. JS); Framework (Django with REST (DRF) API); Git &amp; SDLC; Data Structures &amp; Algorithms (Python); Machine Learning (Supervised &amp; Unsupervised); Artificial Intelligence</t>
+  </si>
+  <si>
+    <t>Frontend (Figma, HTML, CSS, JavaScript); Backend (Core &amp; Advance Java); Frontend Library (React. JS); Framework (Springboot); Git &amp; SDLC; Data Structures &amp; Algorithms (Python)</t>
+  </si>
+  <si>
+    <t>Frontend (Figma, HTML, CSS, JavaScript); Database (Mongo DB); Frontend Library (React. JS); Framework (Node js with REST API); Git &amp; SDLC</t>
+  </si>
+  <si>
+    <t>Frontend (Figma, HTML, CSS, JavaScript); Backend (Core &amp; Advance Java); Frontend Library (React. JS); Framework (Springboot with API); Git &amp; SDLC; Data Structures &amp; Algorithms (Python); Mobile App (Flutter)</t>
+  </si>
+  <si>
+    <t>Frontend (Figma, HTML, CSS, JavaScript); Backend (Core &amp; Advance Java); Framework (Springboot with CRUD); Data Structures &amp; Algorithms (with Java)</t>
+  </si>
+  <si>
+    <t>Frontend (Figma, HTML, CSS, JavaScript); Database (Mongo DB); Frontend Library (React. JS); Framework (Node js with REST API)</t>
+  </si>
+  <si>
+    <t>Frontend (Figma, HTML, CSS, JavaScript); Backend (Core &amp; Advance Python); Frontend Library (React. JS); Framework (Django with REST (DRF) API)</t>
+  </si>
+  <si>
+    <t>Figma, HTML, CSS, JavaScript; Backend (Core &amp; Advance Python); Frontend Library (React. JS); Framework (Django with REST (DRF) API)</t>
+  </si>
+  <si>
+    <t>Foundation; Security Essentials; Ethical Hacking Methodology; Web Application Security; Security Operations &amp; Incident Response; AWS Solution Architect — Security Focus; Advanced VAPT; Mobile &amp; Digital Forensics; Red Team Operations; Bug Bounty &amp; Hacker Mindset; Build Modern Infrastructure; Automate the Platform; AI Foundations for Security Professionals; Generative AI in Practice; AI Agents &amp; AI Security</t>
+  </si>
+  <si>
+    <t>Foundation; Security Essentials; Ethical Hacking Methodology; Web Application Security; Security Operations &amp; Incident Response; AWS Solution Architect — Security Focus; Advanced VAPT; Mobile &amp; Digital Forensics; Red Team Operations; Bug Bounty &amp; Hacker Mindset</t>
+  </si>
+  <si>
+    <t>Foundation; Security Essentials; Ethical Hacking Methodology; Web Application Security; Security Operations &amp; Incident Response</t>
+  </si>
+  <si>
+    <t>Python Fundamentals; Data Structures &amp; Data Fundamentals; Machine Learning Foundations; Data Analytics &amp; Visualization; Computer Vision; AI/ML Foundations &amp; Deep Learning; GenAI Foundations; Vibe Coding / AI-Assisted Development; LLM Application Development; RAG; AI Agents; Advanced Agentic AI; MLOps / AIOps; SQL &amp; Database Management; AWS / Cloud; IoT &amp; Embedded Systems; AI + IoT Integration; Full-Stack Development; AI Product Development; AI Engineering; Robotics &amp; Smart Systems; Deployment &amp; Production; Capstone &amp; Industry Project</t>
+  </si>
+  <si>
+    <t>Python Fundamentals; Machine Learning Foundations; GenAI Foundations; Vibe Coding / AI-Assisted Development; AI Product Development</t>
+  </si>
+  <si>
+    <t>Python Fundamentals; Machine Learning Foundations; Computer Vision; IoT &amp; Embedded Systems; AI + IoT Integration</t>
+  </si>
+  <si>
+    <t>Python Fundamentals; AI/ML Foundations &amp; Deep Learning; GenAI Foundations; LLM Application Development; RAG; AI Agents; Advanced Agentic AI; AWS / Cloud</t>
+  </si>
+  <si>
+    <t>Python Fundamentals; Data Structures &amp; Data Fundamentals; Data Analytics &amp; Visualization; GenAI Foundations; Vibe Coding / AI-Assisted Development; LLM Application Development; RAG; AI Agents; MLOps / AIOps; SQL &amp; Database Management</t>
+  </si>
+  <si>
+    <t>Python Fundamentals; Data Structures &amp; Data Fundamentals; Machine Learning Foundations; Data Analytics &amp; Visualization; AI/ML Foundations &amp; Deep Learning; GenAI Foundations; LLM Application Development; RAG; AI Agents; MLOps / AIOps; AWS / Cloud; IoT &amp; Embedded Systems; AI + IoT Integration</t>
+  </si>
+  <si>
+    <t>Full-Stack Development; AI Product Development; AI Engineering; Robotics &amp; Smart Systems; Deployment &amp; Production; Capstone &amp; Industry Project</t>
+  </si>
+  <si>
+    <t>GenAI Foundations; LLM Application Development; RAG; AI Agents; Advanced Agentic AI; IoT &amp; Embedded Systems; AI + IoT Integration; Full-Stack Development</t>
+  </si>
+  <si>
+    <t>Data Analytics Foundations; Advanced Excel; Statistics for Data Analytics; Python Programming for Analytics; NumPy &amp; Pandas; Data Visualization with Python; SQL &amp; Database Analytics; Power BI &amp; Business Intelligence; Exploratory Data Analysis (EDA); ETL &amp; Data Preparation; Digital Business Analytics; Digital Marketing Analytics; GenAI Tools for Data Analytics; Graphics &amp; Video for Digital Analytics; Advanced Analytics Projects; Industry Internship / Capstone</t>
+  </si>
+  <si>
+    <t>Data Analytics Foundations; Advanced Excel; Statistics for Data Analytics; Python Programming for Analytics; Power BI &amp; Business Intelligence</t>
+  </si>
+  <si>
+    <t>Data Analytics Foundations; Advanced Excel; Statistics for Data Analytics; Python Programming for Analytics; NumPy &amp; Pandas; Data Visualization with Python; SQL &amp; Database Analytics; Power BI &amp; Business Intelligence; Exploratory Data Analysis (EDA); ETL &amp; Data Preparation</t>
+  </si>
+  <si>
+    <t>Digital Marketing Foundations &amp; Strategy; SEO Specialist Track; Website Development &amp; Landing Pages; Social Media Marketing &amp; Management; Content Marketing &amp; Copywriting; Lead Generation, Landing Pages &amp; Conversion; Search Engine Marketing (SEM) &amp; Paid Search; Online Display &amp; Remarketing; E-Commerce &amp; Online Sales Marketing; Video Marketing &amp; YouTube; Mobile App Marketing; Google Ads Ecosystem: Discovery, Performance Max &amp; Search; Growth, Reputation, Email &amp; Messaging; Freelancing, Portfolio, Resume &amp; Interview Readiness; AI-Powered Digital Marketing &amp; Career Growth</t>
+  </si>
+  <si>
+    <t>Digital Marketing Foundations &amp; Strategy; SEO Specialist Track; Website Development &amp; Landing Pages; Social Media Marketing &amp; Management; Content Marketing &amp; Copywriting; Lead Generation, Landing Pages &amp; Conversion; Search Engine Marketing (SEM) &amp; Paid Search; Online Display &amp; Remarketing</t>
+  </si>
+  <si>
+    <t>Digital Marketing Foundations &amp; Strategy; SEO Specialist Track; Website Development &amp; Landing Pages; Social Media Marketing &amp; Management; Content Marketing &amp; Copywriting; Lead Generation, Landing Pages &amp; Conversion; Search Engine Marketing (SEM) &amp; Paid Search; Online Display &amp; Remarketing; E-Commerce &amp; Online Sales Marketing; Video Marketing &amp; YouTube; Mobile App Marketing; Google Ads Ecosystem: Discovery, Performance Max &amp; Search</t>
   </si>
   <si>
     <t>full-stack-data-science-with-ai-course</t>
@@ -780,10 +873,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -823,562 +916,658 @@
       <c r="M1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F2" t="s">
+        <v>115</v>
+      </c>
+      <c r="L2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F3" t="s">
+        <v>116</v>
+      </c>
+      <c r="L3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F5" t="s">
+        <v>118</v>
+      </c>
+      <c r="L5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F6" t="s">
+        <v>119</v>
+      </c>
+      <c r="L6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F7" t="s">
+        <v>120</v>
+      </c>
+      <c r="L7" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
         <v>22</v>
       </c>
-      <c r="D2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E2" t="s">
-        <v>84</v>
-      </c>
-      <c r="K2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" t="s">
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F8" t="s">
+        <v>121</v>
+      </c>
+      <c r="L8" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F9" t="s">
+        <v>122</v>
+      </c>
+      <c r="L9" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" t="s">
+        <v>93</v>
+      </c>
+      <c r="F10" t="s">
+        <v>123</v>
+      </c>
+      <c r="L10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F11" t="s">
+        <v>124</v>
+      </c>
+      <c r="L11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s">
+        <v>64</v>
+      </c>
+      <c r="E12" t="s">
+        <v>95</v>
+      </c>
+      <c r="F12" t="s">
+        <v>125</v>
+      </c>
+      <c r="L12" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" t="s">
+        <v>126</v>
+      </c>
+      <c r="L13" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" t="s">
+        <v>97</v>
+      </c>
+      <c r="F14" t="s">
+        <v>127</v>
+      </c>
+      <c r="L14" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" t="s">
+        <v>98</v>
+      </c>
+      <c r="F15" t="s">
+        <v>128</v>
+      </c>
+      <c r="L15" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" t="s">
+        <v>68</v>
+      </c>
+      <c r="E16" t="s">
+        <v>99</v>
+      </c>
+      <c r="F16" t="s">
+        <v>129</v>
+      </c>
+      <c r="L16" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" t="s">
+        <v>100</v>
+      </c>
+      <c r="F17" t="s">
+        <v>130</v>
+      </c>
+      <c r="L17" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E18" t="s">
+        <v>101</v>
+      </c>
+      <c r="F18" t="s">
+        <v>131</v>
+      </c>
+      <c r="L18" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" t="s">
+        <v>71</v>
+      </c>
+      <c r="E19" t="s">
+        <v>102</v>
+      </c>
+      <c r="F19" t="s">
+        <v>132</v>
+      </c>
+      <c r="L19" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" t="s">
+        <v>103</v>
+      </c>
+      <c r="F20" t="s">
+        <v>133</v>
+      </c>
+      <c r="L20" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" t="s">
+        <v>42</v>
+      </c>
+      <c r="D21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E21" t="s">
+        <v>104</v>
+      </c>
+      <c r="F21" t="s">
+        <v>134</v>
+      </c>
+      <c r="L21" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" t="s">
+        <v>105</v>
+      </c>
+      <c r="F22" t="s">
+        <v>135</v>
+      </c>
+      <c r="L22" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" t="s">
+        <v>75</v>
+      </c>
+      <c r="E23" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23" t="s">
+        <v>136</v>
+      </c>
+      <c r="L23" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" t="s">
+        <v>76</v>
+      </c>
+      <c r="E24" t="s">
+        <v>107</v>
+      </c>
+      <c r="F24" t="s">
+        <v>137</v>
+      </c>
+      <c r="L24" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" t="s">
+        <v>108</v>
+      </c>
+      <c r="F25" t="s">
+        <v>138</v>
+      </c>
+      <c r="L25" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C26" t="s">
+        <v>47</v>
+      </c>
+      <c r="D26" t="s">
+        <v>78</v>
+      </c>
+      <c r="E26" t="s">
+        <v>109</v>
+      </c>
+      <c r="F26" t="s">
+        <v>139</v>
+      </c>
+      <c r="L26" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27" t="s">
+        <v>79</v>
+      </c>
+      <c r="E27" t="s">
+        <v>110</v>
+      </c>
+      <c r="F27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L27" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" t="s">
+        <v>49</v>
+      </c>
+      <c r="D28" t="s">
+        <v>80</v>
+      </c>
+      <c r="E28" t="s">
+        <v>111</v>
+      </c>
+      <c r="F28" t="s">
+        <v>141</v>
+      </c>
+      <c r="L28" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" t="s">
+        <v>81</v>
+      </c>
+      <c r="E29" t="s">
+        <v>109</v>
+      </c>
+      <c r="F29" t="s">
+        <v>142</v>
+      </c>
+      <c r="L29" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E3" t="s">
-        <v>85</v>
-      </c>
-      <c r="K3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E5" t="s">
-        <v>87</v>
-      </c>
-      <c r="K5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E6" t="s">
-        <v>88</v>
-      </c>
-      <c r="K6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" t="s">
-        <v>89</v>
-      </c>
-      <c r="K7" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" t="s">
-        <v>60</v>
-      </c>
-      <c r="E9" t="s">
-        <v>91</v>
-      </c>
-      <c r="K9" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" t="s">
-        <v>61</v>
-      </c>
-      <c r="E10" t="s">
-        <v>92</v>
-      </c>
-      <c r="K10" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" t="s">
-        <v>62</v>
-      </c>
-      <c r="E11" t="s">
-        <v>93</v>
-      </c>
-      <c r="K11" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" t="s">
-        <v>63</v>
-      </c>
-      <c r="E12" t="s">
-        <v>94</v>
-      </c>
-      <c r="K12" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" t="s">
-        <v>64</v>
-      </c>
-      <c r="E13" t="s">
-        <v>95</v>
-      </c>
-      <c r="K13" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" t="s">
-        <v>65</v>
-      </c>
-      <c r="E14" t="s">
-        <v>96</v>
-      </c>
-      <c r="K14" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
-      <c r="A15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" t="s">
-        <v>66</v>
-      </c>
-      <c r="E15" t="s">
-        <v>97</v>
-      </c>
-      <c r="K15" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" t="s">
-        <v>67</v>
-      </c>
-      <c r="E16" t="s">
-        <v>98</v>
-      </c>
-      <c r="K16" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" t="s">
-        <v>37</v>
-      </c>
-      <c r="D17" t="s">
-        <v>68</v>
-      </c>
-      <c r="E17" t="s">
-        <v>99</v>
-      </c>
-      <c r="K17" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
-      <c r="A18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" t="s">
-        <v>38</v>
-      </c>
-      <c r="D18" t="s">
-        <v>69</v>
-      </c>
-      <c r="E18" t="s">
-        <v>100</v>
-      </c>
-      <c r="K18" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11">
-      <c r="A19" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" t="s">
-        <v>70</v>
-      </c>
-      <c r="E19" t="s">
-        <v>101</v>
-      </c>
-      <c r="K19" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11">
-      <c r="A20" t="s">
-        <v>16</v>
-      </c>
-      <c r="C20" t="s">
-        <v>40</v>
-      </c>
-      <c r="D20" t="s">
-        <v>71</v>
-      </c>
-      <c r="E20" t="s">
-        <v>102</v>
-      </c>
-      <c r="K20" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11">
-      <c r="A21" t="s">
-        <v>16</v>
-      </c>
-      <c r="C21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D21" t="s">
-        <v>72</v>
-      </c>
-      <c r="E21" t="s">
-        <v>103</v>
-      </c>
-      <c r="K21" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11">
-      <c r="A22" t="s">
-        <v>16</v>
-      </c>
-      <c r="C22" t="s">
-        <v>42</v>
-      </c>
-      <c r="D22" t="s">
-        <v>73</v>
-      </c>
-      <c r="E22" t="s">
-        <v>104</v>
-      </c>
-      <c r="K22" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11">
-      <c r="A23" t="s">
-        <v>16</v>
-      </c>
-      <c r="C23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" t="s">
-        <v>74</v>
-      </c>
-      <c r="E23" t="s">
-        <v>105</v>
-      </c>
-      <c r="K23" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11">
-      <c r="A24" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" t="s">
-        <v>75</v>
-      </c>
-      <c r="E24" t="s">
-        <v>106</v>
-      </c>
-      <c r="K24" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11">
-      <c r="A25" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" t="s">
-        <v>45</v>
-      </c>
-      <c r="D25" t="s">
-        <v>76</v>
-      </c>
-      <c r="E25" t="s">
-        <v>107</v>
-      </c>
-      <c r="K25" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
-      <c r="A26" t="s">
-        <v>13</v>
-      </c>
-      <c r="C26" t="s">
-        <v>46</v>
-      </c>
-      <c r="D26" t="s">
-        <v>77</v>
-      </c>
-      <c r="E26" t="s">
-        <v>108</v>
-      </c>
-      <c r="K26" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
-      <c r="A27" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" t="s">
-        <v>47</v>
-      </c>
-      <c r="D27" t="s">
-        <v>78</v>
-      </c>
-      <c r="E27" t="s">
-        <v>109</v>
-      </c>
-      <c r="K27" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
-      <c r="A28" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" t="s">
-        <v>48</v>
-      </c>
-      <c r="D28" t="s">
-        <v>79</v>
-      </c>
-      <c r="E28" t="s">
-        <v>110</v>
-      </c>
-      <c r="K28" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11">
-      <c r="A29" t="s">
-        <v>13</v>
-      </c>
-      <c r="C29" t="s">
-        <v>49</v>
-      </c>
-      <c r="D29" t="s">
-        <v>80</v>
-      </c>
-      <c r="E29" t="s">
-        <v>111</v>
-      </c>
-      <c r="K29" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11">
-      <c r="A30" t="s">
-        <v>17</v>
-      </c>
       <c r="C30" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E30" t="s">
         <v>112</v>
       </c>
-      <c r="K30" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11">
+      <c r="F30" t="s">
+        <v>143</v>
+      </c>
+      <c r="L30" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
       <c r="A31" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C31" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D31" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E31" t="s">
         <v>113</v>
       </c>
-      <c r="K31" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11">
+      <c r="F31" t="s">
+        <v>144</v>
+      </c>
+      <c r="L31" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
       <c r="A32" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C32" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D32" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E32" t="s">
         <v>114</v>
       </c>
-      <c r="K32" t="s">
-        <v>144</v>
+      <c r="F32" t="s">
+        <v>145</v>
+      </c>
+      <c r="L32" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>